<commit_message>
Refactorizacion cientifica Q1: validacion espacial, Nested CV, SMOTENC, Macro F1, econometria espacial y reportes automaticos
</commit_message>
<xml_diff>
--- a/outputs/metrics/model_comparison_metrics.xlsx
+++ b/outputs/metrics/model_comparison_metrics.xlsx
@@ -7,80 +7,104 @@
     <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
   </bookViews>
   <sheets>
-    <sheet name="Performance Metrics" sheetId="1" r:id="rId1"/>
+    <sheet name="Metrics" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="20">
-  <si>
-    <t>Model</t>
-  </si>
-  <si>
-    <t>Accuracy</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="28">
+  <si>
+    <t>Modelo</t>
+  </si>
+  <si>
+    <t>Macro F1 (Principal)</t>
   </si>
   <si>
     <t>Balanced Accuracy</t>
   </si>
   <si>
+    <t>Recall (Macro)</t>
+  </si>
+  <si>
+    <t>MCC Multiclase</t>
+  </si>
+  <si>
     <t>Precision (Macro)</t>
   </si>
   <si>
-    <t>Precision (Weighted)</t>
-  </si>
-  <si>
-    <t>Recall (Macro)</t>
-  </si>
-  <si>
-    <t>Recall (Weighted)</t>
-  </si>
-  <si>
-    <t>F1 (Macro)</t>
-  </si>
-  <si>
-    <t>F1 (Weighted)</t>
-  </si>
-  <si>
-    <t>Sensitivity (Macro)</t>
-  </si>
-  <si>
-    <t>Specificity (Macro)</t>
-  </si>
-  <si>
-    <t>MCC</t>
-  </si>
-  <si>
-    <t>Cohen Kappa</t>
-  </si>
-  <si>
-    <t>ROC AUC</t>
+    <t>ROC-AUC (OvR)</t>
+  </si>
+  <si>
+    <t>PR-AUC (OvR)</t>
+  </si>
+  <si>
+    <t>Accuracy (Secundario)</t>
   </si>
   <si>
     <t>Log Loss</t>
   </si>
   <si>
-    <t>Train Time (s)</t>
-  </si>
-  <si>
-    <t>Prediction Time (s)</t>
-  </si>
-  <si>
-    <t>Regresión Logística</t>
-  </si>
-  <si>
-    <t>XGBoost</t>
-  </si>
-  <si>
-    <t>G-XGBoost Espacial</t>
+    <t>Tiempo Entrenamiento (s)</t>
+  </si>
+  <si>
+    <t>Tiempo Predicción (s)</t>
+  </si>
+  <si>
+    <t>Recall_Arma Blanca</t>
+  </si>
+  <si>
+    <t>Precision_Arma Blanca</t>
+  </si>
+  <si>
+    <t>F1_Arma Blanca</t>
+  </si>
+  <si>
+    <t>Recall_Arma de Fuego</t>
+  </si>
+  <si>
+    <t>Precision_Arma de Fuego</t>
+  </si>
+  <si>
+    <t>F1_Arma de Fuego</t>
+  </si>
+  <si>
+    <t>Recall_Otros</t>
+  </si>
+  <si>
+    <t>Precision_Otros</t>
+  </si>
+  <si>
+    <t>F1_Otros</t>
+  </si>
+  <si>
+    <t>XGBoost con Covariables Geográficas</t>
+  </si>
+  <si>
+    <t>Extra Trees</t>
+  </si>
+  <si>
+    <t>Random Forest</t>
+  </si>
+  <si>
+    <t>XGBoost Base (No Espacial)</t>
+  </si>
+  <si>
+    <t>Regresión Logística Multinomial</t>
+  </si>
+  <si>
+    <t>Baseline Territorial (Parroquia)</t>
+  </si>
+  <si>
+    <t>Baseline Clase Mayoritaria</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -88,30 +112,16 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFD7E4BC"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -119,30 +129,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -437,219 +429,527 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:Q4"/>
+  <dimension ref="A1:U8"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:17">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
+    <row r="1" spans="1:21">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" t="s">
         <v>16</v>
       </c>
+      <c r="R1" t="s">
+        <v>17</v>
+      </c>
+      <c r="S1" t="s">
+        <v>18</v>
+      </c>
+      <c r="T1" t="s">
+        <v>19</v>
+      </c>
+      <c r="U1" t="s">
+        <v>20</v>
+      </c>
     </row>
-    <row r="2" spans="1:17">
+    <row r="2" spans="1:21">
       <c r="A2" t="s">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="B2">
-        <v>0.6270462633451958</v>
+        <v>0.415636500916931</v>
       </c>
       <c r="C2">
-        <v>0.458120198789461</v>
+        <v>0.4718964985668575</v>
       </c>
       <c r="D2">
-        <v>0.3852495978160191</v>
+        <v>0.4718964985668575</v>
       </c>
       <c r="E2">
-        <v>0.8478263762256137</v>
+        <v>0.220065112356121</v>
       </c>
       <c r="F2">
-        <v>0.458120198789461</v>
+        <v>0.4099119665639425</v>
       </c>
       <c r="G2">
-        <v>0.6270462633451958</v>
+        <v>0.7443924672495768</v>
       </c>
       <c r="H2">
-        <v>0.3687670480207246</v>
+        <v>0.4102093036230596</v>
       </c>
       <c r="I2">
-        <v>0.7081914307279161</v>
+        <v>0.7902149740548554</v>
       </c>
       <c r="J2">
-        <v>0.458120198789461</v>
+        <v>0.6583301424980164</v>
       </c>
       <c r="K2">
-        <v>0.7734783018834577</v>
+        <v>0.3721182346343994</v>
       </c>
       <c r="L2">
-        <v>0.1572772263583066</v>
+        <v>0.02445554733276367</v>
       </c>
       <c r="M2">
-        <v>0.1233002644793828</v>
+        <v>0.4347826086956522</v>
       </c>
       <c r="N2">
-        <v>0.6843239285319621</v>
+        <v>0.1449275362318841</v>
       </c>
       <c r="O2">
-        <v>0.8874401831329761</v>
+        <v>0.2173913043478261</v>
       </c>
       <c r="P2">
-        <v>0.3107054233551025</v>
+        <v>0.8405560098119379</v>
       </c>
       <c r="Q2">
-        <v>0.0005645751953125</v>
+        <v>0.9492151431209603</v>
+      </c>
+      <c r="R2">
+        <v>0.8915871639202082</v>
+      </c>
+      <c r="S2">
+        <v>0.1403508771929824</v>
+      </c>
+      <c r="T2">
+        <v>0.1355932203389831</v>
+      </c>
+      <c r="U2">
+        <v>0.1379310344827586</v>
       </c>
     </row>
-    <row r="3" spans="1:17">
+    <row r="3" spans="1:21">
       <c r="A3" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="B3">
-        <v>0.8768683274021353</v>
+        <v>0.3996728772752858</v>
       </c>
       <c r="C3">
-        <v>0.4483904717492285</v>
+        <v>0.3856337313118197</v>
       </c>
       <c r="D3">
-        <v>0.5364205102246105</v>
+        <v>0.3856337313118197</v>
       </c>
       <c r="E3">
-        <v>0.8493849686028612</v>
+        <v>0.1516583542051638</v>
       </c>
       <c r="F3">
-        <v>0.4483904717492285</v>
+        <v>0.5404681923157674</v>
       </c>
       <c r="G3">
-        <v>0.8768683274021353</v>
+        <v>0.619033615228572</v>
       </c>
       <c r="H3">
-        <v>0.4749618798311255</v>
+        <v>0.3924510671977853</v>
       </c>
       <c r="I3">
-        <v>0.8595314693823051</v>
+        <v>0.8917716827279466</v>
       </c>
       <c r="J3">
-        <v>0.4483904717492285</v>
+        <v>0.4975808672548777</v>
       </c>
       <c r="K3">
-        <v>0.7428116629483549</v>
+        <v>0.4036483764648438</v>
       </c>
       <c r="L3">
-        <v>0.2642150047682552</v>
+        <v>0.08715009689331055</v>
       </c>
       <c r="M3">
-        <v>0.2516978529779387</v>
+        <v>0.1304347826086956</v>
       </c>
       <c r="N3">
-        <v>0.7076587041923598</v>
+        <v>0.2045454545454546</v>
       </c>
       <c r="O3">
-        <v>0.4623809446583384</v>
+        <v>0.1592920353982301</v>
       </c>
       <c r="P3">
-        <v>1.199063301086426</v>
+        <v>0.9738348323793949</v>
       </c>
       <c r="Q3">
-        <v>0.006325483322143555</v>
+        <v>0.9168591224018475</v>
+      </c>
+      <c r="R3">
+        <v>0.9444885011895321</v>
+      </c>
+      <c r="S3">
+        <v>0.05263157894736842</v>
+      </c>
+      <c r="T3">
+        <v>0.5</v>
+      </c>
+      <c r="U3">
+        <v>0.09523809523809523</v>
       </c>
     </row>
-    <row r="4" spans="1:17">
+    <row r="4" spans="1:21">
       <c r="A4" t="s">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="B4">
-        <v>0.9039145907473309</v>
+        <v>0.387971280162078</v>
       </c>
       <c r="C4">
-        <v>0.514925680426348</v>
+        <v>0.3768627370267184</v>
       </c>
       <c r="D4">
-        <v>0.7021360899954514</v>
+        <v>0.3768627370267184</v>
       </c>
       <c r="E4">
-        <v>0.8841231232326343</v>
+        <v>0.1517030656024935</v>
       </c>
       <c r="F4">
-        <v>0.514925680426348</v>
+        <v>0.4672990083562116</v>
       </c>
       <c r="G4">
-        <v>0.9039145907473309</v>
+        <v>0.7037839348131886</v>
       </c>
       <c r="H4">
-        <v>0.568894587912676</v>
+        <v>0.4172374189475268</v>
       </c>
       <c r="I4">
-        <v>0.8863962504710661</v>
+        <v>0.8954781319495922</v>
       </c>
       <c r="J4">
-        <v>0.514925680426348</v>
+        <v>0.3827449936991343</v>
       </c>
       <c r="K4">
-        <v>0.7709417708934674</v>
+        <v>0.4440031051635742</v>
       </c>
       <c r="L4">
-        <v>0.4169427822438446</v>
+        <v>0.06436896324157715</v>
       </c>
       <c r="M4">
-        <v>0.3850864623384707</v>
+        <v>0.1159420289855072</v>
       </c>
       <c r="N4">
-        <v>0.8105449844548982</v>
+        <v>0.2352941176470588</v>
       </c>
       <c r="O4">
-        <v>0.3649207862110065</v>
+        <v>0.1553398058252427</v>
       </c>
       <c r="P4">
-        <v>1.90351128578186</v>
+        <v>0.9795584627964022</v>
       </c>
       <c r="Q4">
-        <v>0.007853031158447266</v>
+        <v>0.9166029074215761</v>
+      </c>
+      <c r="R4">
+        <v>0.9470355731225296</v>
+      </c>
+      <c r="S4">
+        <v>0.03508771929824561</v>
+      </c>
+      <c r="T4">
+        <v>0.25</v>
+      </c>
+      <c r="U4">
+        <v>0.06153846153846154</v>
+      </c>
+    </row>
+    <row r="5" spans="1:21">
+      <c r="A5" t="s">
+        <v>24</v>
+      </c>
+      <c r="B5">
+        <v>0.3432432771200887</v>
+      </c>
+      <c r="C5">
+        <v>0.4346021535286781</v>
+      </c>
+      <c r="D5">
+        <v>0.4346021535286781</v>
+      </c>
+      <c r="E5">
+        <v>0.1345556109279555</v>
+      </c>
+      <c r="F5">
+        <v>0.3670070977086777</v>
+      </c>
+      <c r="G5">
+        <v>0.6988878935872544</v>
+      </c>
+      <c r="H5">
+        <v>0.4045615505984379</v>
+      </c>
+      <c r="I5">
+        <v>0.6419570051890289</v>
+      </c>
+      <c r="J5">
+        <v>0.8047587871551514</v>
+      </c>
+      <c r="K5">
+        <v>0.2462525367736816</v>
+      </c>
+      <c r="L5">
+        <v>0.01843905448913574</v>
+      </c>
+      <c r="M5">
+        <v>0.5072463768115942</v>
+      </c>
+      <c r="N5">
+        <v>0.100864553314121</v>
+      </c>
+      <c r="O5">
+        <v>0.1682692307692308</v>
+      </c>
+      <c r="P5">
+        <v>0.6737530662305805</v>
+      </c>
+      <c r="Q5">
+        <v>0.9471264367816092</v>
+      </c>
+      <c r="R5">
+        <v>0.7873865265169613</v>
+      </c>
+      <c r="S5">
+        <v>0.1228070175438596</v>
+      </c>
+      <c r="T5">
+        <v>0.05303030303030303</v>
+      </c>
+      <c r="U5">
+        <v>0.07407407407407407</v>
+      </c>
+    </row>
+    <row r="6" spans="1:21">
+      <c r="A6" t="s">
+        <v>25</v>
+      </c>
+      <c r="B6">
+        <v>0.3265576913014732</v>
+      </c>
+      <c r="C6">
+        <v>0.4447594093960177</v>
+      </c>
+      <c r="D6">
+        <v>0.4447594093960177</v>
+      </c>
+      <c r="E6">
+        <v>0.1251817259440968</v>
+      </c>
+      <c r="F6">
+        <v>0.3669737581472228</v>
+      </c>
+      <c r="G6">
+        <v>0.6679168240341458</v>
+      </c>
+      <c r="H6">
+        <v>0.3866405353823736</v>
+      </c>
+      <c r="I6">
+        <v>0.5744996293550778</v>
+      </c>
+      <c r="J6">
+        <v>0.969726295729061</v>
+      </c>
+      <c r="K6">
+        <v>0.1800799369812012</v>
+      </c>
+      <c r="L6">
+        <v>0.01330661773681641</v>
+      </c>
+      <c r="M6">
+        <v>0.5652173913043478</v>
+      </c>
+      <c r="N6">
+        <v>0.09725685785536159</v>
+      </c>
+      <c r="O6">
+        <v>0.1659574468085106</v>
+      </c>
+      <c r="P6">
+        <v>0.5936222403924775</v>
+      </c>
+      <c r="Q6">
+        <v>0.9490196078431372</v>
+      </c>
+      <c r="R6">
+        <v>0.7303822937625755</v>
+      </c>
+      <c r="S6">
+        <v>0.1754385964912281</v>
+      </c>
+      <c r="T6">
+        <v>0.0546448087431694</v>
+      </c>
+      <c r="U6">
+        <v>0.08333333333333333</v>
+      </c>
+    </row>
+    <row r="7" spans="1:21">
+      <c r="A7" t="s">
+        <v>26</v>
+      </c>
+      <c r="B7">
+        <v>0.3170036288232245</v>
+      </c>
+      <c r="C7">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="D7">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="E7">
+        <v>0</v>
+      </c>
+      <c r="F7">
+        <v>0.3021991598715097</v>
+      </c>
+      <c r="G7">
+        <v>0.5</v>
+      </c>
+      <c r="H7">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="I7">
+        <v>0.9065974796145293</v>
+      </c>
+      <c r="J7">
+        <v>3.366568070443856</v>
+      </c>
+      <c r="K7">
+        <v>0.01113128662109375</v>
+      </c>
+      <c r="L7">
+        <v>0.001782655715942383</v>
+      </c>
+      <c r="M7">
+        <v>0</v>
+      </c>
+      <c r="N7">
+        <v>0</v>
+      </c>
+      <c r="O7">
+        <v>0</v>
+      </c>
+      <c r="P7">
+        <v>1</v>
+      </c>
+      <c r="Q7">
+        <v>0.9065974796145293</v>
+      </c>
+      <c r="R7">
+        <v>0.9510108864696734</v>
+      </c>
+      <c r="S7">
+        <v>0</v>
+      </c>
+      <c r="T7">
+        <v>0</v>
+      </c>
+      <c r="U7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:21">
+      <c r="A8" t="s">
+        <v>27</v>
+      </c>
+      <c r="B8">
+        <v>0.3170036288232245</v>
+      </c>
+      <c r="C8">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="D8">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="E8">
+        <v>0</v>
+      </c>
+      <c r="F8">
+        <v>0.3021991598715097</v>
+      </c>
+      <c r="G8">
+        <v>0.5</v>
+      </c>
+      <c r="H8">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="I8">
+        <v>0.9065974796145293</v>
+      </c>
+      <c r="J8">
+        <v>3.366568070443856</v>
+      </c>
+      <c r="K8">
+        <v>0.002260923385620117</v>
+      </c>
+      <c r="L8">
+        <v>0.0003564357757568359</v>
+      </c>
+      <c r="M8">
+        <v>0</v>
+      </c>
+      <c r="N8">
+        <v>0</v>
+      </c>
+      <c r="O8">
+        <v>0</v>
+      </c>
+      <c r="P8">
+        <v>1</v>
+      </c>
+      <c r="Q8">
+        <v>0.9065974796145293</v>
+      </c>
+      <c r="R8">
+        <v>0.9510108864696734</v>
+      </c>
+      <c r="S8">
+        <v>0</v>
+      </c>
+      <c r="T8">
+        <v>0</v>
+      </c>
+      <c r="U8">
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Informe de Auditoria Cientifica Q1 y mejoras de evaluacion
</commit_message>
<xml_diff>
--- a/outputs/metrics/model_comparison_metrics.xlsx
+++ b/outputs/metrics/model_comparison_metrics.xlsx
@@ -529,10 +529,10 @@
         <v>0.6583301424980164</v>
       </c>
       <c r="K2">
-        <v>0.3721182346343994</v>
+        <v>0.2831490039825439</v>
       </c>
       <c r="L2">
-        <v>0.02445554733276367</v>
+        <v>0.01512765884399414</v>
       </c>
       <c r="M2">
         <v>0.4347826086956522</v>
@@ -594,10 +594,10 @@
         <v>0.4975808672548777</v>
       </c>
       <c r="K3">
-        <v>0.4036483764648438</v>
+        <v>0.404062032699585</v>
       </c>
       <c r="L3">
-        <v>0.08715009689331055</v>
+        <v>0.0681915283203125</v>
       </c>
       <c r="M3">
         <v>0.1304347826086956</v>
@@ -659,10 +659,10 @@
         <v>0.3827449936991343</v>
       </c>
       <c r="K4">
-        <v>0.4440031051635742</v>
+        <v>0.4068689346313477</v>
       </c>
       <c r="L4">
-        <v>0.06436896324157715</v>
+        <v>0.06644797325134277</v>
       </c>
       <c r="M4">
         <v>0.1159420289855072</v>
@@ -724,10 +724,10 @@
         <v>0.8047587871551514</v>
       </c>
       <c r="K5">
-        <v>0.2462525367736816</v>
+        <v>0.1524162292480469</v>
       </c>
       <c r="L5">
-        <v>0.01843905448913574</v>
+        <v>0.01700639724731445</v>
       </c>
       <c r="M5">
         <v>0.5072463768115942</v>
@@ -789,10 +789,10 @@
         <v>0.969726295729061</v>
       </c>
       <c r="K6">
-        <v>0.1800799369812012</v>
+        <v>0.1307473182678223</v>
       </c>
       <c r="L6">
-        <v>0.01330661773681641</v>
+        <v>0.007755756378173828</v>
       </c>
       <c r="M6">
         <v>0.5652173913043478</v>
@@ -854,10 +854,10 @@
         <v>3.366568070443856</v>
       </c>
       <c r="K7">
-        <v>0.01113128662109375</v>
+        <v>0.01709771156311035</v>
       </c>
       <c r="L7">
-        <v>0.001782655715942383</v>
+        <v>0.002440214157104492</v>
       </c>
       <c r="M7">
         <v>0</v>
@@ -919,10 +919,10 @@
         <v>3.366568070443856</v>
       </c>
       <c r="K8">
-        <v>0.002260923385620117</v>
+        <v>0.001275062561035156</v>
       </c>
       <c r="L8">
-        <v>0.0003564357757568359</v>
+        <v>0.0002858638763427734</v>
       </c>
       <c r="M8">
         <v>0</v>

</xml_diff>